<commit_message>
paper run 2026-10-30 10:22
</commit_message>
<xml_diff>
--- a/reports/2026-10-30.xlsx
+++ b/reports/2026-10-30.xlsx
@@ -681,13 +681,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C15" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D15" t="n">
-        <v>574.23</v>
+        <v>756.78</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
@@ -700,13 +700,13 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C16" t="n">
         <v>3</v>
       </c>
       <c r="D16" t="n">
-        <v>352.67</v>
+        <v>167.44</v>
       </c>
       <c r="E16" t="n">
         <v>18.55</v>
@@ -764,13 +764,13 @@
         </is>
       </c>
       <c r="B20" t="n">
+        <v>5</v>
+      </c>
+      <c r="C20" t="n">
         <v>3</v>
       </c>
-      <c r="C20" t="n">
-        <v>2</v>
-      </c>
       <c r="D20" t="n">
-        <v>144.53</v>
+        <v>141.85</v>
       </c>
       <c r="E20" t="n">
         <v>0</v>
@@ -809,13 +809,13 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C23" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D23" t="n">
-        <v>592.95</v>
+        <v>775.5</v>
       </c>
       <c r="E23" t="n">
         <v>0</v>
@@ -847,13 +847,13 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C25" t="n">
         <v>2</v>
       </c>
       <c r="D25" t="n">
-        <v>257.4</v>
+        <v>72.17</v>
       </c>
       <c r="E25" t="n">
         <v>0</v>
@@ -873,13 +873,13 @@
         </is>
       </c>
       <c r="B27" t="n">
+        <v>9</v>
+      </c>
+      <c r="C27" t="n">
         <v>7</v>
       </c>
-      <c r="C27" t="n">
-        <v>6</v>
-      </c>
       <c r="D27" t="n">
-        <v>789.88</v>
+        <v>787.2</v>
       </c>
       <c r="E27" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
paper run 2026-10-30 17:56
</commit_message>
<xml_diff>
--- a/reports/2026-10-30.xlsx
+++ b/reports/2026-10-30.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -515,6 +515,221 @@
       </c>
       <c r="K2" t="n">
         <v>18.55</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-10-30T13:54:12.764889+00:00</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>5</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="F3" t="n">
+        <v>31</v>
+      </c>
+      <c r="G3" t="n">
+        <v>50</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.805</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.00174</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K3" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-10-30T14:24:03.517886+00:00</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>5</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="F4" t="n">
+        <v>2.55</v>
+      </c>
+      <c r="G4" t="n">
+        <v>5</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.775</v>
+      </c>
+      <c r="I4" t="n">
+        <v>-0.00105</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
+        <v>2.45</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-10-30T15:54:29.848674+00:00</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ETH</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>5</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="F5" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="G5" t="n">
+        <v>20</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.804</v>
+      </c>
+      <c r="I5" t="n">
+        <v>-0.00115</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>9.199999999999999</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-10-30T16:11:17.180002+00:00</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ETH</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>15</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="F6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="G6" t="n">
+        <v>10</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.793</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.00224</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
+        <v>3.9</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-10-30T17:11:16.006813+00:00</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>15</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.6158</v>
+      </c>
+      <c r="F7" t="n">
+        <v>36.95</v>
+      </c>
+      <c r="G7" t="n">
+        <v>60</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="I7" t="n">
+        <v>-0.00148</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K7" t="n">
+        <v>23.05</v>
       </c>
     </row>
   </sheetData>
@@ -528,7 +743,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E48"/>
+  <dimension ref="A1:E63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -550,7 +765,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3">
@@ -560,7 +775,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4">
@@ -590,7 +805,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>18.55</v>
+        <v>76.15000000000001</v>
       </c>
     </row>
     <row r="7">
@@ -600,7 +815,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>18.55</v>
+        <v>76.15000000000001</v>
       </c>
     </row>
     <row r="8">
@@ -630,7 +845,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>4285.959999999999</v>
+        <v>4343.559999999999</v>
       </c>
     </row>
     <row r="12">
@@ -681,16 +896,16 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C15" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D15" t="n">
-        <v>756.78</v>
+        <v>1516.08</v>
       </c>
       <c r="E15" t="n">
-        <v>0</v>
+        <v>26.95</v>
       </c>
     </row>
     <row r="16">
@@ -700,16 +915,16 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="C16" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="D16" t="n">
-        <v>167.44</v>
+        <v>1583.39</v>
       </c>
       <c r="E16" t="n">
-        <v>18.55</v>
+        <v>49.2</v>
       </c>
     </row>
     <row r="17">
@@ -726,13 +941,13 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D18" t="n">
-        <v>213.37</v>
+        <v>412.17</v>
       </c>
       <c r="E18" t="n">
         <v>0</v>
@@ -745,16 +960,16 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="C19" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="D19" t="n">
-        <v>267.8</v>
+        <v>1030.95</v>
       </c>
       <c r="E19" t="n">
-        <v>18.55</v>
+        <v>31.65</v>
       </c>
     </row>
     <row r="20">
@@ -764,16 +979,16 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C20" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="D20" t="n">
-        <v>141.85</v>
+        <v>1042.15</v>
       </c>
       <c r="E20" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
     </row>
     <row r="21">
@@ -783,16 +998,16 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C21" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D21" t="n">
-        <v>301.2</v>
+        <v>614.2</v>
       </c>
       <c r="E21" t="n">
-        <v>0</v>
+        <v>25.5</v>
       </c>
     </row>
     <row r="22">
@@ -809,16 +1024,16 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="C23" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="D23" t="n">
-        <v>775.5</v>
+        <v>2346.29</v>
       </c>
       <c r="E23" t="n">
-        <v>0</v>
+        <v>11.65</v>
       </c>
     </row>
     <row r="24">
@@ -847,16 +1062,16 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="C25" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="D25" t="n">
-        <v>72.17</v>
+        <v>676.63</v>
       </c>
       <c r="E25" t="n">
-        <v>0</v>
+        <v>45.95</v>
       </c>
     </row>
     <row r="26">
@@ -869,17 +1084,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>NO_LIQUIDITY</t>
+          <t>MAX_PER_WINDOW</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="C27" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="D27" t="n">
-        <v>787.2</v>
+        <v>583.8099999999999</v>
       </c>
       <c r="E27" t="n">
         <v>0</v>
@@ -888,109 +1103,122 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
+          <t>NO_LIQUIDITY</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>14</v>
+      </c>
+      <c r="C28" t="n">
+        <v>12</v>
+      </c>
+      <c r="D28" t="n">
+        <v>1621.64</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="B28" t="n">
-        <v>1</v>
-      </c>
-      <c r="C28" t="n">
-        <v>1</v>
-      </c>
-      <c r="D28" t="n">
-        <v>137.02</v>
-      </c>
-      <c r="E28" t="n">
-        <v>18.55</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
+      <c r="B29" t="n">
+        <v>6</v>
+      </c>
+      <c r="C29" t="n">
+        <v>6</v>
+      </c>
+      <c r="D29" t="n">
+        <v>894.02</v>
+      </c>
+      <c r="E29" t="n">
+        <v>76.15000000000001</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
         <is>
           <t>REALIZED (реальные сделки)</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>По активам</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
+          <t>По активам</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
           <t>ETH</t>
         </is>
       </c>
-      <c r="B33" t="n">
-        <v>1</v>
-      </c>
-      <c r="C33" t="n">
-        <v>1</v>
-      </c>
-      <c r="D33" t="n">
-        <v>18.55</v>
+      <c r="B34" t="n">
+        <v>3</v>
+      </c>
+      <c r="C34" t="n">
+        <v>3</v>
+      </c>
+      <c r="D34" t="n">
+        <v>31.65</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>По окнам</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>1</v>
+      </c>
+      <c r="C35" t="n">
+        <v>1</v>
+      </c>
+      <c r="D35" t="n">
+        <v>19</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>5m</t>
+          <t>XRP</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C36" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D36" t="n">
-        <v>18.55</v>
+        <v>25.5</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>По часам</t>
+          <t>По окнам</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1012,83 +1240,93 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>15m</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C39" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D39" t="n">
-        <v>18.55</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>По цене входа</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+        <v>26.95</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>5m</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>4</v>
+      </c>
+      <c r="C40" t="n">
+        <v>4</v>
+      </c>
+      <c r="D40" t="n">
+        <v>49.2</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>0.55–0.60</t>
-        </is>
-      </c>
-      <c r="B42" t="n">
-        <v>1</v>
-      </c>
-      <c r="C42" t="n">
-        <v>1</v>
-      </c>
-      <c r="D42" t="n">
+          <t>По часам</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>1</v>
+      </c>
+      <c r="C43" t="n">
+        <v>1</v>
+      </c>
+      <c r="D43" t="n">
         <v>18.55</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>По силе движения</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>1</v>
+      </c>
+      <c r="C44" t="n">
+        <v>1</v>
+      </c>
+      <c r="D44" t="n">
+        <v>19</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>0.12–0.15%</t>
+          <t>14</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1098,45 +1336,265 @@
         <v>1</v>
       </c>
       <c r="D45" t="n">
-        <v>18.55</v>
+        <v>2.45</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>1</v>
+      </c>
+      <c r="C46" t="n">
+        <v>1</v>
+      </c>
+      <c r="D46" t="n">
+        <v>9.199999999999999</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>По направлению</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>1</v>
+      </c>
+      <c r="C47" t="n">
+        <v>1</v>
+      </c>
+      <c r="D47" t="n">
+        <v>3.9</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>1</v>
+      </c>
+      <c r="C48" t="n">
+        <v>1</v>
+      </c>
+      <c r="D48" t="n">
+        <v>23.05</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>По цене входа</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>0.50–0.55</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>2</v>
+      </c>
+      <c r="C51" t="n">
+        <v>2</v>
+      </c>
+      <c r="D51" t="n">
+        <v>11.65</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>0.55–0.60</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>1</v>
+      </c>
+      <c r="C52" t="n">
+        <v>1</v>
+      </c>
+      <c r="D52" t="n">
+        <v>18.55</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>0.60–0.62</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>3</v>
+      </c>
+      <c r="C53" t="n">
+        <v>3</v>
+      </c>
+      <c r="D53" t="n">
+        <v>45.95</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>По силе движения</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>0.10–0.12%</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>2</v>
+      </c>
+      <c r="C56" t="n">
+        <v>2</v>
+      </c>
+      <c r="D56" t="n">
+        <v>11.65</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>0.12–0.15%</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>2</v>
+      </c>
+      <c r="C57" t="n">
+        <v>2</v>
+      </c>
+      <c r="D57" t="n">
+        <v>41.6</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>0.15–0.20%</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>1</v>
+      </c>
+      <c r="C58" t="n">
+        <v>1</v>
+      </c>
+      <c r="D58" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>0.20%+</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>1</v>
+      </c>
+      <c r="C59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D59" t="n">
+        <v>3.9</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>По направлению</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
           <t>DOWN</t>
         </is>
       </c>
-      <c r="B48" t="n">
-        <v>1</v>
-      </c>
-      <c r="C48" t="n">
-        <v>1</v>
-      </c>
-      <c r="D48" t="n">
-        <v>18.55</v>
+      <c r="B62" t="n">
+        <v>4</v>
+      </c>
+      <c r="C62" t="n">
+        <v>4</v>
+      </c>
+      <c r="D62" t="n">
+        <v>53.25</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>2</v>
+      </c>
+      <c r="C63" t="n">
+        <v>2</v>
+      </c>
+      <c r="D63" t="n">
+        <v>22.9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>